<commit_message>
Fix project list export function
</commit_message>
<xml_diff>
--- a/src/main/resources/template/ProjectList.xlsx
+++ b/src/main/resources/template/ProjectList.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hyuntae.you\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\FOSSLight\work\2026\OSC-5217 enterprise 소스코드 업로드\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34385A08-68E7-411F-AD75-4EB2E9F5E244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="120" windowWidth="16152" windowHeight="11436"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -41,96 +42,64 @@
     <t>Project Name</t>
   </si>
   <si>
-    <t>Software Version</t>
+    <t>Reviewer</t>
+  </si>
+  <si>
+    <t>Packaging</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Status</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Identification</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSC Process</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Distribution</t>
-  </si>
-  <si>
-    <t>Reviewer</t>
-  </si>
-  <si>
-    <t>Packaging</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Status</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Status</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Source Code</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>BIN</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Description</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Site</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Last Deployed</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Master Category</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Notice Type</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Operating System</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Status</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>3rd party</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Identification</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>BOM (Disclose)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Notice File</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Pakage File</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Models</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>CVSS Score</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Download</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fosslight
+Report</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSS Notice</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>OSS
+Packaging</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Security</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Priority</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Modified Date</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,12 +134,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -278,7 +241,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -288,16 +251,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -338,7 +295,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -355,9 +312,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -395,9 +352,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -432,7 +389,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -467,7 +424,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -640,146 +597,96 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z3"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.69921875" customWidth="1"/>
-    <col min="2" max="2" width="10.09765625" customWidth="1"/>
-    <col min="3" max="3" width="24.8984375" customWidth="1"/>
-    <col min="4" max="4" width="16.3984375" customWidth="1"/>
-    <col min="5" max="5" width="23.59765625" customWidth="1"/>
-    <col min="6" max="6" width="20.3984375" customWidth="1"/>
-    <col min="8" max="11" width="11" customWidth="1"/>
-    <col min="13" max="13" width="27.09765625" customWidth="1"/>
-    <col min="14" max="14" width="40.09765625" customWidth="1"/>
-    <col min="15" max="15" width="39.3984375" customWidth="1"/>
-    <col min="16" max="16" width="12.09765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.09765625" customWidth="1"/>
-    <col min="18" max="18" width="30.59765625" customWidth="1"/>
-    <col min="19" max="19" width="21.59765625" customWidth="1"/>
-    <col min="20" max="20" width="42.09765625" customWidth="1"/>
-    <col min="21" max="21" width="15.59765625" customWidth="1"/>
-    <col min="22" max="23" width="20.3984375" customWidth="1"/>
-    <col min="25" max="25" width="13.69921875" customWidth="1"/>
-    <col min="26" max="26" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.75" customWidth="1"/>
+    <col min="2" max="2" width="24.875" customWidth="1"/>
+    <col min="3" max="3" width="10.125" customWidth="1"/>
+    <col min="4" max="9" width="13.625" customWidth="1"/>
+    <col min="10" max="12" width="20.375" customWidth="1"/>
+    <col min="15" max="16" width="13.75" customWidth="1"/>
+    <col min="17" max="17" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:17" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="6"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="6"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="7" t="s">
+    </row>
+    <row r="2" spans="1:17" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="9"/>
-      <c r="P1" s="6" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
-      <c r="U1" s="6"/>
-      <c r="V1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="F2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
     </row>
-    <row r="2" spans="1:26" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5"/>
-      <c r="Z2" s="5"/>
-    </row>
-    <row r="3" spans="1:26" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:17" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -797,32 +704,22 @@
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="1"/>
-      <c r="U3" s="1"/>
-      <c r="V3" s="1"/>
-      <c r="W3" s="1"/>
-      <c r="X3" s="1"/>
-      <c r="Y3" s="1"/>
-      <c r="Z3" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="Z1:Z2"/>
-    <mergeCell ref="V1:V2"/>
+  <mergeCells count="13">
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="L1:L2"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="C1:C2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="W1:W2"/>
-    <mergeCell ref="X1:X2"/>
-    <mergeCell ref="Y1:Y2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="P1:U1"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="L1:O1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:I1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -831,9 +728,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -841,9 +738,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>